<commit_message>
Almost finished data scrapper
</commit_message>
<xml_diff>
--- a/main/Rezultate_Cazari.xlsx
+++ b/main/Rezultate_Cazari.xlsx
@@ -31,6 +31,9 @@
     <x:t>Descriere</x:t>
   </x:si>
   <x:si>
+    <x:t>Imagine</x:t>
+  </x:si>
+  <x:si>
     <x:t>AnuntCazare</x:t>
   </x:si>
   <x:si>
@@ -46,10 +49,19 @@
     <x:t>Cameră comună în Barcelona</x:t>
   </x:si>
   <x:si>
+    <x:t>97 lei</x:t>
+  </x:si>
+  <x:si>
+    <x:t>4,71</x:t>
+  </x:si>
+  <x:si>
+    <x:t>https://www.airbnb.com.ro/rooms/1381830149578594250?adults=1&amp;check_in=2026-02-01&amp;check_out=2026-02-02&amp;search_mode=regular_search&amp;source_impression_id=p3_1767620337_P3ENn5ggIUoNBGN2&amp;previous_page_section_name=1000&amp;federated_search_id=01800970-e477-43d9-8377-6c604c3bf98a</x:t>
+  </x:si>
+  <x:si>
     <x:t/>
   </x:si>
   <x:si>
-    <x:t>4,71</x:t>
+    <x:t>https://a0.muscache.com/im/pictures/hosting/Hosting-U3RheVN1cHBseUxpc3Rpbmc6MTM4MTgzMDE0OTU3ODU5NDI1MA==/original/69db4bfd-4e0d-41f7-be36-6c7668b3a34c.jpeg?im_w=720</x:t>
   </x:si>
   <x:si>
     <x:t>Locuință din topul categoriei Alegerea oaspeților
@@ -70,19 +82,19 @@
 4,71 (301)</x:t>
   </x:si>
   <x:si>
-    <x:t>97 lei</x:t>
-  </x:si>
-  <x:si>
-    <x:t>https://www.airbnb.com.ro/rooms/1381830149578594250?adults=1&amp;check_in=2026-02-01&amp;check_out=2026-02-02&amp;search_mode=regular_search&amp;source_impression_id=p3_1767620337_P3ENn5ggIUoNBGN2&amp;previous_page_section_name=1000&amp;federated_search_id=01800970-e477-43d9-8377-6c604c3bf98a</x:t>
-  </x:si>
-  <x:si>
-    <x:t>https://a0.muscache.com/im/pictures/hosting/Hosting-U3RheVN1cHBseUxpc3Rpbmc6MTM4MTgzMDE0OTU3ODU5NDI1MA==/original/69db4bfd-4e0d-41f7-be36-6c7668b3a34c.jpeg?im_w=720</x:t>
-  </x:si>
-  <x:si>
     <x:t>Hostel în Barcelona</x:t>
   </x:si>
   <x:si>
+    <x:t>362 lei</x:t>
+  </x:si>
+  <x:si>
     <x:t>4,75</x:t>
+  </x:si>
+  <x:si>
+    <x:t>https://www.airbnb.com.ro/rooms/52047123?adults=1&amp;check_in=2026-02-01&amp;check_out=2026-02-02&amp;search_mode=regular_search&amp;source_impression_id=p3_1767620337_P3UTafn9rFGC5_Uz&amp;previous_page_section_name=1000&amp;federated_search_id=01800970-e477-43d9-8377-6c604c3bf98a</x:t>
+  </x:si>
+  <x:si>
+    <x:t>https://a0.muscache.com/im/pictures/a039d4f3-bcf6-4d60-84c8-e8391b271be7.jpg?im_w=720</x:t>
   </x:si>
   <x:si>
     <x:t>Alegerea oaspeților
@@ -104,19 +116,19 @@
 4,75 (413)</x:t>
   </x:si>
   <x:si>
-    <x:t>362 lei</x:t>
-  </x:si>
-  <x:si>
-    <x:t>https://www.airbnb.com.ro/rooms/52047123?adults=1&amp;check_in=2026-02-01&amp;check_out=2026-02-02&amp;search_mode=regular_search&amp;source_impression_id=p3_1767620337_P3UTafn9rFGC5_Uz&amp;previous_page_section_name=1000&amp;federated_search_id=01800970-e477-43d9-8377-6c604c3bf98a</x:t>
-  </x:si>
-  <x:si>
-    <x:t>https://a0.muscache.com/im/pictures/a039d4f3-bcf6-4d60-84c8-e8391b271be7.jpg?im_w=720</x:t>
-  </x:si>
-  <x:si>
     <x:t>Cazare în Barcelona</x:t>
   </x:si>
   <x:si>
+    <x:t>171 lei</x:t>
+  </x:si>
+  <x:si>
     <x:t>4,77</x:t>
+  </x:si>
+  <x:si>
+    <x:t>https://www.airbnb.com.ro/rooms/1150749414787336366?adults=1&amp;check_in=2026-02-01&amp;check_out=2026-02-02&amp;search_mode=regular_search&amp;source_impression_id=p3_1767620337_P3xydsiprI-PNH1_&amp;previous_page_section_name=1000&amp;federated_search_id=01800970-e477-43d9-8377-6c604c3bf98a</x:t>
+  </x:si>
+  <x:si>
+    <x:t>https://a0.muscache.com/im/pictures/miso/Hosting-1150749414787336366/original/229baae8-0bf6-475e-aecb-e6ddfc731dba.jpeg?im_w=720</x:t>
   </x:si>
   <x:si>
     <x:t>Cazare în Barcelona
@@ -135,16 +147,16 @@
 4,77 (13)</x:t>
   </x:si>
   <x:si>
-    <x:t>171 lei</x:t>
-  </x:si>
-  <x:si>
-    <x:t>https://www.airbnb.com.ro/rooms/1150749414787336366?adults=1&amp;check_in=2026-02-01&amp;check_out=2026-02-02&amp;search_mode=regular_search&amp;source_impression_id=p3_1767620337_P3xydsiprI-PNH1_&amp;previous_page_section_name=1000&amp;federated_search_id=01800970-e477-43d9-8377-6c604c3bf98a</x:t>
-  </x:si>
-  <x:si>
-    <x:t>https://a0.muscache.com/im/pictures/miso/Hosting-1150749414787336366/original/229baae8-0bf6-475e-aecb-e6ddfc731dba.jpeg?im_w=720</x:t>
+    <x:t>330 lei</x:t>
   </x:si>
   <x:si>
     <x:t>4,9</x:t>
+  </x:si>
+  <x:si>
+    <x:t>https://www.airbnb.com.ro/rooms/1517954062359728775?adults=1&amp;check_in=2026-02-01&amp;check_out=2026-02-02&amp;search_mode=regular_search&amp;source_impression_id=p3_1767620337_P3LGwNgJkFjV5Tcb&amp;previous_page_section_name=1000&amp;federated_search_id=01800970-e477-43d9-8377-6c604c3bf98a</x:t>
+  </x:si>
+  <x:si>
+    <x:t>https://a0.muscache.com/im/pictures/hosting/Hosting-1517954062359728775/original/5c0ed819-27d6-480a-aa25-64a4a6fc79ee.jpeg?im_w=720</x:t>
   </x:si>
   <x:si>
     <x:t>Cazare în Barcelona
@@ -163,16 +175,13 @@
 4,9 (10)</x:t>
   </x:si>
   <x:si>
-    <x:t>330 lei</x:t>
-  </x:si>
-  <x:si>
-    <x:t>https://www.airbnb.com.ro/rooms/1517954062359728775?adults=1&amp;check_in=2026-02-01&amp;check_out=2026-02-02&amp;search_mode=regular_search&amp;source_impression_id=p3_1767620337_P3LGwNgJkFjV5Tcb&amp;previous_page_section_name=1000&amp;federated_search_id=01800970-e477-43d9-8377-6c604c3bf98a</x:t>
-  </x:si>
-  <x:si>
-    <x:t>https://a0.muscache.com/im/pictures/hosting/Hosting-1517954062359728775/original/5c0ed819-27d6-480a-aa25-64a4a6fc79ee.jpeg?im_w=720</x:t>
-  </x:si>
-  <x:si>
     <x:t>4,8</x:t>
+  </x:si>
+  <x:si>
+    <x:t>https://www.airbnb.com.ro/rooms/45906714?adults=1&amp;check_in=2026-02-01&amp;check_out=2026-02-02&amp;search_mode=regular_search&amp;source_impression_id=p3_1767620337_P3aVRf-1d9tjAXkp&amp;previous_page_section_name=1000&amp;federated_search_id=01800970-e477-43d9-8377-6c604c3bf98a</x:t>
+  </x:si>
+  <x:si>
+    <x:t>https://a0.muscache.com/im/pictures/prohost-api/Hosting-45906714/original/cabe89e2-49ac-4031-ba0a-599b061e0656.jpeg?im_w=720</x:t>
   </x:si>
   <x:si>
     <x:t>Alegerea oaspeților
@@ -194,16 +203,19 @@
 4,8 (46)</x:t>
   </x:si>
   <x:si>
-    <x:t>https://www.airbnb.com.ro/rooms/45906714?adults=1&amp;check_in=2026-02-01&amp;check_out=2026-02-02&amp;search_mode=regular_search&amp;source_impression_id=p3_1767620337_P3aVRf-1d9tjAXkp&amp;previous_page_section_name=1000&amp;federated_search_id=01800970-e477-43d9-8377-6c604c3bf98a</x:t>
-  </x:si>
-  <x:si>
-    <x:t>https://a0.muscache.com/im/pictures/prohost-api/Hosting-45906714/original/cabe89e2-49ac-4031-ba0a-599b061e0656.jpeg?im_w=720</x:t>
-  </x:si>
-  <x:si>
     <x:t>Cameră de hotel în Barcelona</x:t>
   </x:si>
   <x:si>
+    <x:t>506 lei</x:t>
+  </x:si>
+  <x:si>
     <x:t>4,7</x:t>
+  </x:si>
+  <x:si>
+    <x:t>https://www.airbnb.com.ro/rooms/32931496?adults=1&amp;check_in=2026-02-01&amp;check_out=2026-02-02&amp;search_mode=regular_search&amp;source_impression_id=p3_1767620337_P3Fd9342xxdSBDM-&amp;previous_page_section_name=1000&amp;federated_search_id=01800970-e477-43d9-8377-6c604c3bf98a</x:t>
+  </x:si>
+  <x:si>
+    <x:t>https://a0.muscache.com/im/pictures/miso/Hosting-32931496/original/eb34add6-434d-4724-8fed-edd2d32cd9d6.jpeg?im_w=720</x:t>
   </x:si>
   <x:si>
     <x:t>Super-gazdă
@@ -224,19 +236,16 @@
 4,7 (271)</x:t>
   </x:si>
   <x:si>
-    <x:t>506 lei</x:t>
-  </x:si>
-  <x:si>
-    <x:t>https://www.airbnb.com.ro/rooms/32931496?adults=1&amp;check_in=2026-02-01&amp;check_out=2026-02-02&amp;search_mode=regular_search&amp;source_impression_id=p3_1767620337_P3Fd9342xxdSBDM-&amp;previous_page_section_name=1000&amp;federated_search_id=01800970-e477-43d9-8377-6c604c3bf98a</x:t>
-  </x:si>
-  <x:si>
-    <x:t>https://a0.muscache.com/im/pictures/miso/Hosting-32931496/original/eb34add6-434d-4724-8fed-edd2d32cd9d6.jpeg?im_w=720</x:t>
-  </x:si>
-  <x:si>
-    <x:t>366 lei</x:t>
+    <x:t>83 lei</x:t>
   </x:si>
   <x:si>
     <x:t>4,44</x:t>
+  </x:si>
+  <x:si>
+    <x:t>https://www.airbnb.com.ro/rooms/1395616579066520047?adults=1&amp;check_in=2026-02-01&amp;check_out=2026-02-02&amp;search_mode=regular_search&amp;source_impression_id=p3_1767620337_P3Nc4sAvY9AHthhE&amp;previous_page_section_name=1000&amp;federated_search_id=01800970-e477-43d9-8377-6c604c3bf98a</x:t>
+  </x:si>
+  <x:si>
+    <x:t>https://a0.muscache.com/im/pictures/miso/Hosting-52981104/original/295fae11-18ea-4ab1-af39-aa3448fd6e87.jpeg?im_w=720</x:t>
   </x:si>
   <x:si>
     <x:t>Cameră comună în Barcelona
@@ -256,19 +265,19 @@
 4,44 (870)</x:t>
   </x:si>
   <x:si>
-    <x:t>83 lei</x:t>
-  </x:si>
-  <x:si>
-    <x:t>https://www.airbnb.com.ro/rooms/1395616579066520047?adults=1&amp;check_in=2026-02-01&amp;check_out=2026-02-02&amp;search_mode=regular_search&amp;source_impression_id=p3_1767620337_P3Nc4sAvY9AHthhE&amp;previous_page_section_name=1000&amp;federated_search_id=01800970-e477-43d9-8377-6c604c3bf98a</x:t>
-  </x:si>
-  <x:si>
-    <x:t>https://a0.muscache.com/im/pictures/miso/Hosting-52981104/original/295fae11-18ea-4ab1-af39-aa3448fd6e87.jpeg?im_w=720</x:t>
-  </x:si>
-  <x:si>
     <x:t>Hotel în Barcelona</x:t>
   </x:si>
   <x:si>
+    <x:t>436 lei</x:t>
+  </x:si>
+  <x:si>
     <x:t>4,64</x:t>
+  </x:si>
+  <x:si>
+    <x:t>https://www.airbnb.com.ro/rooms/1440590229528643742?adults=1&amp;check_in=2026-02-01&amp;check_out=2026-02-02&amp;search_mode=regular_search&amp;source_impression_id=p3_1767620337_P3OCnUmDohuFgJMM&amp;previous_page_section_name=1000&amp;federated_search_id=01800970-e477-43d9-8377-6c604c3bf98a</x:t>
+  </x:si>
+  <x:si>
+    <x:t>https://a0.muscache.com/im/pictures/prohost-api/Hosting-1440590229528643742/original/711aea61-aad9-4bd7-8063-450fd11ae5e1.jpeg?im_w=720</x:t>
   </x:si>
   <x:si>
     <x:t>Hotel în Barcelona
@@ -287,16 +296,16 @@
 4,64 (166)</x:t>
   </x:si>
   <x:si>
-    <x:t>436 lei</x:t>
-  </x:si>
-  <x:si>
-    <x:t>https://www.airbnb.com.ro/rooms/1440590229528643742?adults=1&amp;check_in=2026-02-01&amp;check_out=2026-02-02&amp;search_mode=regular_search&amp;source_impression_id=p3_1767620337_P3OCnUmDohuFgJMM&amp;previous_page_section_name=1000&amp;federated_search_id=01800970-e477-43d9-8377-6c604c3bf98a</x:t>
-  </x:si>
-  <x:si>
-    <x:t>https://a0.muscache.com/im/pictures/prohost-api/Hosting-1440590229528643742/original/711aea61-aad9-4bd7-8063-450fd11ae5e1.jpeg?im_w=720</x:t>
+    <x:t>275 lei</x:t>
   </x:si>
   <x:si>
     <x:t>4,88</x:t>
+  </x:si>
+  <x:si>
+    <x:t>https://www.airbnb.com.ro/rooms/1537621078010972051?adults=1&amp;check_in=2026-02-01&amp;check_out=2026-02-02&amp;search_mode=regular_search&amp;source_impression_id=p3_1767620337_P3DI5UkM4gJb6ioQ&amp;previous_page_section_name=1000&amp;federated_search_id=01800970-e477-43d9-8377-6c604c3bf98a</x:t>
+  </x:si>
+  <x:si>
+    <x:t>https://a0.muscache.com/im/pictures/hosting/Hosting-1537621078010972051/original/76f324a0-7c43-4842-bce5-93c777917b6a.jpeg?im_w=720</x:t>
   </x:si>
   <x:si>
     <x:t>Alegerea oaspeților
@@ -318,56 +327,19 @@
 4,88 (16)</x:t>
   </x:si>
   <x:si>
-    <x:t>275 lei</x:t>
-  </x:si>
-  <x:si>
-    <x:t>https://www.airbnb.com.ro/rooms/1537621078010972051?adults=1&amp;check_in=2026-02-01&amp;check_out=2026-02-02&amp;search_mode=regular_search&amp;source_impression_id=p3_1767620337_P3DI5UkM4gJb6ioQ&amp;previous_page_section_name=1000&amp;federated_search_id=01800970-e477-43d9-8377-6c604c3bf98a</x:t>
-  </x:si>
-  <x:si>
-    <x:t>https://a0.muscache.com/im/pictures/hosting/Hosting-1537621078010972051/original/76f324a0-7c43-4842-bce5-93c777917b6a.jpeg?im_w=720</x:t>
-  </x:si>
-  <x:si>
-    <x:t>710</x:t>
-  </x:si>
-  <x:si>
-    <x:t>4,74</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Alegerea oaspeților
-Alegerea oaspeților
-710
-Recenzii
-4,74
-Stele
-Scor
-9
-Ani de experiență ca gazdă
-Cameră în L'Hospitalet de Llobregat
-Hogar Coris gat@ , este posibil să existe păr viu
-1 pat de o persoană
-1 pat de o persoană
-Gazdă persoană fizică
-Gazdă persoană fizică
-196 lei
-Afișează defalcarea prețului
-pentru 1 noapte
-Scor mediu de 4,74 din 5, 710 recenzii
-4,74 (710)</x:t>
-  </x:si>
-  <x:si>
-    <x:t>196 lei</x:t>
-  </x:si>
-  <x:si>
-    <x:t>https://www.airbnb.com.ro/rooms/15924643?adults=1&amp;check_in=2026-02-01&amp;check_out=2026-02-02&amp;search_mode=regular_search&amp;category_tag=Tag%3A8678&amp;photo_id=2006904328&amp;source_impression_id=p3_1767620337_P376YN1VcCWE4EqX&amp;previous_page_section_name=1000&amp;federated_search_id=01800970-e477-43d9-8377-6c604c3bf98a</x:t>
-  </x:si>
-  <x:si>
-    <x:t>https://a0.muscache.com/im/pictures/hosting/Hosting-15924643/original/339c5cbe-547d-4136-9798-d3ce52eee5a5.jpeg?im_w=720</x:t>
-  </x:si>
-  <x:si>
     <x:t>Cameră în L'Hospitalet de Llobregat</x:t>
   </x:si>
   <x:si>
+    <x:t>214 lei</x:t>
+  </x:si>
+  <x:si>
     <x:t>4,78</x:t>
+  </x:si>
+  <x:si>
+    <x:t>https://www.airbnb.com.ro/rooms/1205592108295952981?adults=1&amp;check_in=2026-02-01&amp;check_out=2026-02-02&amp;search_mode=regular_search&amp;category_tag=Tag%3A8678&amp;photo_id=1957747260&amp;source_impression_id=p3_1767620337_P3tGQPUBvaLZBkgf&amp;previous_page_section_name=1000&amp;federated_search_id=01800970-e477-43d9-8377-6c604c3bf98a</x:t>
+  </x:si>
+  <x:si>
+    <x:t>https://a0.muscache.com/im/pictures/hosting/Hosting-1205592108295952981/original/4ff62bd9-ffc4-48cb-8fc8-6cf1ca5aab0a.jpeg?im_w=720</x:t>
   </x:si>
   <x:si>
     <x:t>Cameră în L'Hospitalet de Llobregat
@@ -383,19 +355,19 @@
 4,78 (130)</x:t>
   </x:si>
   <x:si>
-    <x:t>214 lei</x:t>
-  </x:si>
-  <x:si>
-    <x:t>https://www.airbnb.com.ro/rooms/1205592108295952981?adults=1&amp;check_in=2026-02-01&amp;check_out=2026-02-02&amp;search_mode=regular_search&amp;category_tag=Tag%3A8678&amp;photo_id=1957747260&amp;source_impression_id=p3_1767620337_P3tGQPUBvaLZBkgf&amp;previous_page_section_name=1000&amp;federated_search_id=01800970-e477-43d9-8377-6c604c3bf98a</x:t>
-  </x:si>
-  <x:si>
-    <x:t>https://a0.muscache.com/im/pictures/hosting/Hosting-1205592108295952981/original/4ff62bd9-ffc4-48cb-8fc8-6cf1ca5aab0a.jpeg?im_w=720</x:t>
-  </x:si>
-  <x:si>
     <x:t>Pensiune cu mic dejun în Barcelona</x:t>
   </x:si>
   <x:si>
+    <x:t>376 lei</x:t>
+  </x:si>
+  <x:si>
     <x:t>4,6</x:t>
+  </x:si>
+  <x:si>
+    <x:t>https://www.airbnb.com.ro/rooms/1027571829045048978?adults=1&amp;check_in=2026-02-01&amp;check_out=2026-02-02&amp;search_mode=regular_search&amp;source_impression_id=p3_1767620337_P3WBUFGO1S-8JoIL&amp;previous_page_section_name=1000&amp;federated_search_id=01800970-e477-43d9-8377-6c604c3bf98a</x:t>
+  </x:si>
+  <x:si>
+    <x:t>https://a0.muscache.com/im/pictures/miso/Hosting-1027571829045048978/original/77a6d923-bba2-4972-a507-b8f2f8e03f33.jpeg?im_w=720</x:t>
   </x:si>
   <x:si>
     <x:t>Pensiune cu mic dejun în Barcelona
@@ -414,13 +386,13 @@
 4,6 (99)</x:t>
   </x:si>
   <x:si>
-    <x:t>376 lei</x:t>
-  </x:si>
-  <x:si>
-    <x:t>https://www.airbnb.com.ro/rooms/1027571829045048978?adults=1&amp;check_in=2026-02-01&amp;check_out=2026-02-02&amp;search_mode=regular_search&amp;source_impression_id=p3_1767620337_P3WBUFGO1S-8JoIL&amp;previous_page_section_name=1000&amp;federated_search_id=01800970-e477-43d9-8377-6c604c3bf98a</x:t>
-  </x:si>
-  <x:si>
-    <x:t>https://a0.muscache.com/im/pictures/miso/Hosting-1027571829045048978/original/77a6d923-bba2-4972-a507-b8f2f8e03f33.jpeg?im_w=720</x:t>
+    <x:t>107 lei</x:t>
+  </x:si>
+  <x:si>
+    <x:t>https://www.airbnb.com.ro/rooms/1081106888283937930?adults=1&amp;check_in=2026-02-01&amp;check_out=2026-02-02&amp;search_mode=regular_search&amp;source_impression_id=p3_1767620337_P3IU1WeMFJFU4Ukp&amp;previous_page_section_name=1000&amp;federated_search_id=01800970-e477-43d9-8377-6c604c3bf98a</x:t>
+  </x:si>
+  <x:si>
+    <x:t>https://a0.muscache.com/im/pictures/miso/Hosting-1081106888283937930/original/8eccf776-f01b-4608-93c5-ca469476ef26.jpeg?im_w=720</x:t>
   </x:si>
   <x:si>
     <x:t>Cameră comună în Barcelona
@@ -441,16 +413,16 @@
 4,64 (182)</x:t>
   </x:si>
   <x:si>
-    <x:t>107 lei</x:t>
-  </x:si>
-  <x:si>
-    <x:t>https://www.airbnb.com.ro/rooms/1081106888283937930?adults=1&amp;check_in=2026-02-01&amp;check_out=2026-02-02&amp;search_mode=regular_search&amp;source_impression_id=p3_1767620337_P3IU1WeMFJFU4Ukp&amp;previous_page_section_name=1000&amp;federated_search_id=01800970-e477-43d9-8377-6c604c3bf98a</x:t>
-  </x:si>
-  <x:si>
-    <x:t>https://a0.muscache.com/im/pictures/miso/Hosting-1081106888283937930/original/8eccf776-f01b-4608-93c5-ca469476ef26.jpeg?im_w=720</x:t>
+    <x:t>280 lei</x:t>
   </x:si>
   <x:si>
     <x:t>4,83</x:t>
+  </x:si>
+  <x:si>
+    <x:t>https://www.airbnb.com.ro/rooms/903310566793153888?adults=1&amp;check_in=2026-02-01&amp;check_out=2026-02-02&amp;search_mode=regular_search&amp;category_tag=Tag%3A8678&amp;photo_id=2058915977&amp;source_impression_id=p3_1767620337_P3lERmrsT82YuMgU&amp;previous_page_section_name=1000&amp;federated_search_id=01800970-e477-43d9-8377-6c604c3bf98a</x:t>
+  </x:si>
+  <x:si>
+    <x:t>https://a0.muscache.com/im/pictures/hosting/Hosting-903310566793153888/original/00f1f316-2e9f-4872-8138-657704d412e1.jpeg?im_w=720</x:t>
   </x:si>
   <x:si>
     <x:t>Super-gazdă
@@ -469,16 +441,16 @@
 4,83 (240)</x:t>
   </x:si>
   <x:si>
-    <x:t>280 lei</x:t>
-  </x:si>
-  <x:si>
-    <x:t>https://www.airbnb.com.ro/rooms/903310566793153888?adults=1&amp;check_in=2026-02-01&amp;check_out=2026-02-02&amp;search_mode=regular_search&amp;category_tag=Tag%3A8678&amp;photo_id=2058915977&amp;source_impression_id=p3_1767620337_P3lERmrsT82YuMgU&amp;previous_page_section_name=1000&amp;federated_search_id=01800970-e477-43d9-8377-6c604c3bf98a</x:t>
-  </x:si>
-  <x:si>
-    <x:t>https://a0.muscache.com/im/pictures/hosting/Hosting-903310566793153888/original/00f1f316-2e9f-4872-8138-657704d412e1.jpeg?im_w=720</x:t>
+    <x:t>358 lei</x:t>
   </x:si>
   <x:si>
     <x:t>4,53</x:t>
+  </x:si>
+  <x:si>
+    <x:t>https://www.airbnb.com.ro/rooms/40577359?adults=1&amp;check_in=2026-02-01&amp;check_out=2026-02-02&amp;search_mode=regular_search&amp;source_impression_id=p3_1767620337_P3CnxAWwu0Qh0kzB&amp;previous_page_section_name=1000&amp;federated_search_id=01800970-e477-43d9-8377-6c604c3bf98a</x:t>
+  </x:si>
+  <x:si>
+    <x:t>https://a0.muscache.com/im/pictures/c9f80f52-9b2a-45a7-8822-699255af2338.jpg?im_w=720</x:t>
   </x:si>
   <x:si>
     <x:t>Hotel în Barcelona
@@ -497,13 +469,13 @@
 4,53 (153)</x:t>
   </x:si>
   <x:si>
-    <x:t>358 lei</x:t>
-  </x:si>
-  <x:si>
-    <x:t>https://www.airbnb.com.ro/rooms/40577359?adults=1&amp;check_in=2026-02-01&amp;check_out=2026-02-02&amp;search_mode=regular_search&amp;source_impression_id=p3_1767620337_P3CnxAWwu0Qh0kzB&amp;previous_page_section_name=1000&amp;federated_search_id=01800970-e477-43d9-8377-6c604c3bf98a</x:t>
-  </x:si>
-  <x:si>
-    <x:t>https://a0.muscache.com/im/pictures/c9f80f52-9b2a-45a7-8822-699255af2338.jpg?im_w=720</x:t>
+    <x:t>88 lei</x:t>
+  </x:si>
+  <x:si>
+    <x:t>https://www.airbnb.com.ro/rooms/53602699?adults=1&amp;check_in=2026-02-01&amp;check_out=2026-02-02&amp;search_mode=regular_search&amp;source_impression_id=p3_1767620337_P3KaNAtrmJOwgE2P&amp;previous_page_section_name=1000&amp;federated_search_id=01800970-e477-43d9-8377-6c604c3bf98a</x:t>
+  </x:si>
+  <x:si>
+    <x:t>https://a0.muscache.com/im/pictures/prohost-api/Hosting-53602699/original/2b4a30bd-8cb3-4a46-bf25-afd6a8833b4b.jpeg?im_w=720</x:t>
   </x:si>
   <x:si>
     <x:t>Cameră comună în Barcelona
@@ -523,19 +495,19 @@
 4,7 (10)</x:t>
   </x:si>
   <x:si>
-    <x:t>88 lei</x:t>
-  </x:si>
-  <x:si>
-    <x:t>https://www.airbnb.com.ro/rooms/53602699?adults=1&amp;check_in=2026-02-01&amp;check_out=2026-02-02&amp;search_mode=regular_search&amp;source_impression_id=p3_1767620337_P3KaNAtrmJOwgE2P&amp;previous_page_section_name=1000&amp;federated_search_id=01800970-e477-43d9-8377-6c604c3bf98a</x:t>
-  </x:si>
-  <x:si>
-    <x:t>https://a0.muscache.com/im/pictures/prohost-api/Hosting-53602699/original/2b4a30bd-8cb3-4a46-bf25-afd6a8833b4b.jpeg?im_w=720</x:t>
-  </x:si>
-  <x:si>
     <x:t>Cazare în Premià de Mar</x:t>
   </x:si>
   <x:si>
+    <x:t>251 lei</x:t>
+  </x:si>
+  <x:si>
     <x:t>5,0</x:t>
+  </x:si>
+  <x:si>
+    <x:t>https://www.airbnb.com.ro/rooms/1571042415553002204?adults=1&amp;check_in=2026-02-01&amp;check_out=2026-02-02&amp;search_mode=regular_search&amp;source_impression_id=p3_1767620337_P3cIg9iTuj46QvUg&amp;previous_page_section_name=1000&amp;federated_search_id=01800970-e477-43d9-8377-6c604c3bf98a</x:t>
+  </x:si>
+  <x:si>
+    <x:t>https://a0.muscache.com/im/pictures/hosting/Hosting-1571042415553002204/original/5761d475-f93a-43b8-a713-6ba4135c5033.jpeg?im_w=720</x:t>
   </x:si>
   <x:si>
     <x:t>Cazare în Premià de Mar
@@ -555,16 +527,16 @@
 5,0 (3)</x:t>
   </x:si>
   <x:si>
-    <x:t>251 lei</x:t>
-  </x:si>
-  <x:si>
-    <x:t>https://www.airbnb.com.ro/rooms/1571042415553002204?adults=1&amp;check_in=2026-02-01&amp;check_out=2026-02-02&amp;search_mode=regular_search&amp;source_impression_id=p3_1767620337_P3cIg9iTuj46QvUg&amp;previous_page_section_name=1000&amp;federated_search_id=01800970-e477-43d9-8377-6c604c3bf98a</x:t>
-  </x:si>
-  <x:si>
-    <x:t>https://a0.muscache.com/im/pictures/hosting/Hosting-1571042415553002204/original/5761d475-f93a-43b8-a713-6ba4135c5033.jpeg?im_w=720</x:t>
+    <x:t>448 lei</x:t>
   </x:si>
   <x:si>
     <x:t>4,89</x:t>
+  </x:si>
+  <x:si>
+    <x:t>https://www.airbnb.com.ro/rooms/1133085221552132236?adults=1&amp;check_in=2026-02-01&amp;check_out=2026-02-02&amp;search_mode=regular_search&amp;source_impression_id=p3_1767620337_P3LoaVO0_dwxQ9lR&amp;previous_page_section_name=1000&amp;federated_search_id=01800970-e477-43d9-8377-6c604c3bf98a</x:t>
+  </x:si>
+  <x:si>
+    <x:t>https://a0.muscache.com/im/pictures/prohost-api/Hosting-1133085221552132236/original/e3e56a49-644f-4b03-b633-cb4a05395250.jpeg?im_w=720</x:t>
   </x:si>
   <x:si>
     <x:t>Alegerea oaspeților
@@ -583,18 +555,6 @@
 pentru 1 noapte
 Scor mediu de 4,89 din 5, 81 recenzii
 4,89 (81)</x:t>
-  </x:si>
-  <x:si>
-    <x:t>448 lei</x:t>
-  </x:si>
-  <x:si>
-    <x:t>https://www.airbnb.com.ro/rooms/1133085221552132236?adults=1&amp;check_in=2026-02-01&amp;check_out=2026-02-02&amp;search_mode=regular_search&amp;source_impression_id=p3_1767620337_P3LoaVO0_dwxQ9lR&amp;previous_page_section_name=1000&amp;federated_search_id=01800970-e477-43d9-8377-6c604c3bf98a</x:t>
-  </x:si>
-  <x:si>
-    <x:t>https://a0.muscache.com/im/pictures/prohost-api/Hosting-1133085221552132236/original/e3e56a49-644f-4b03-b633-cb4a05395250.jpeg?im_w=720</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Imagine</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -965,48 +925,48 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="F1" s="0" t="s">
-        <x:v>107</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="G1" s="0" t="s">
-        <x:v>5</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="H1" s="0" t="s">
-        <x:v>6</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="I1" s="0" t="s">
-        <x:v>7</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="J1" s="0" t="s">
-        <x:v>8</x:v>
+        <x:v>9</x:v>
       </x:c>
     </x:row>
     <x:row r="2" spans="1:10">
       <x:c r="A2" s="0" t="s">
-        <x:v>9</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="B2" s="0" t="s">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="C2" s="0" t="s">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="D2" s="0" t="s">
         <x:v>13</x:v>
       </x:c>
-      <x:c r="C2" s="0" t="s">
-        <x:v>11</x:v>
-      </x:c>
-      <x:c r="D2" s="0" t="s">
-        <x:v>14</x:v>
-      </x:c>
       <x:c r="E2" s="0" t="s">
-        <x:v>10</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="F2" s="0" t="s">
         <x:v>15</x:v>
       </x:c>
       <x:c r="G2" s="0" t="s">
-        <x:v>12</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="H2" s="0" t="s">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="I2" s="0" t="s">
         <x:v>13</x:v>
-      </x:c>
-      <x:c r="I2" s="0" t="s">
-        <x:v>14</x:v>
       </x:c>
       <x:c r="J2" s="0" t="s">
         <x:v>15</x:v>
@@ -1014,28 +974,28 @@
     </x:row>
     <x:row r="3" spans="1:10">
       <x:c r="A3" s="0" t="s">
-        <x:v>16</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="B3" s="0" t="s">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="C3" s="0" t="s">
         <x:v>19</x:v>
-      </x:c>
-      <x:c r="C3" s="0" t="s">
-        <x:v>17</x:v>
       </x:c>
       <x:c r="D3" s="0" t="s">
         <x:v>20</x:v>
       </x:c>
       <x:c r="E3" s="0" t="s">
-        <x:v>10</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="F3" s="0" t="s">
         <x:v>21</x:v>
       </x:c>
       <x:c r="G3" s="0" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="H3" s="0" t="s">
         <x:v>18</x:v>
-      </x:c>
-      <x:c r="H3" s="0" t="s">
-        <x:v>19</x:v>
       </x:c>
       <x:c r="I3" s="0" t="s">
         <x:v>20</x:v>
@@ -1046,28 +1006,28 @@
     </x:row>
     <x:row r="4" spans="1:10">
       <x:c r="A4" s="0" t="s">
-        <x:v>22</x:v>
+        <x:v>23</x:v>
       </x:c>
       <x:c r="B4" s="0" t="s">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="C4" s="0" t="s">
         <x:v>25</x:v>
-      </x:c>
-      <x:c r="C4" s="0" t="s">
-        <x:v>23</x:v>
       </x:c>
       <x:c r="D4" s="0" t="s">
         <x:v>26</x:v>
       </x:c>
       <x:c r="E4" s="0" t="s">
-        <x:v>10</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="F4" s="0" t="s">
         <x:v>27</x:v>
       </x:c>
       <x:c r="G4" s="0" t="s">
+        <x:v>28</x:v>
+      </x:c>
+      <x:c r="H4" s="0" t="s">
         <x:v>24</x:v>
-      </x:c>
-      <x:c r="H4" s="0" t="s">
-        <x:v>25</x:v>
       </x:c>
       <x:c r="I4" s="0" t="s">
         <x:v>26</x:v>
@@ -1078,28 +1038,28 @@
     </x:row>
     <x:row r="5" spans="1:10">
       <x:c r="A5" s="0" t="s">
-        <x:v>22</x:v>
+        <x:v>23</x:v>
       </x:c>
       <x:c r="B5" s="0" t="s">
+        <x:v>29</x:v>
+      </x:c>
+      <x:c r="C5" s="0" t="s">
         <x:v>30</x:v>
-      </x:c>
-      <x:c r="C5" s="0" t="s">
-        <x:v>28</x:v>
       </x:c>
       <x:c r="D5" s="0" t="s">
         <x:v>31</x:v>
       </x:c>
       <x:c r="E5" s="0" t="s">
-        <x:v>10</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="F5" s="0" t="s">
         <x:v>32</x:v>
       </x:c>
       <x:c r="G5" s="0" t="s">
+        <x:v>33</x:v>
+      </x:c>
+      <x:c r="H5" s="0" t="s">
         <x:v>29</x:v>
-      </x:c>
-      <x:c r="H5" s="0" t="s">
-        <x:v>30</x:v>
       </x:c>
       <x:c r="I5" s="0" t="s">
         <x:v>31</x:v>
@@ -1110,28 +1070,28 @@
     </x:row>
     <x:row r="6" spans="1:10">
       <x:c r="A6" s="0" t="s">
-        <x:v>9</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="B6" s="0" t="s">
-        <x:v>13</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="C6" s="0" t="s">
-        <x:v>33</x:v>
+        <x:v>34</x:v>
       </x:c>
       <x:c r="D6" s="0" t="s">
         <x:v>35</x:v>
       </x:c>
       <x:c r="E6" s="0" t="s">
-        <x:v>10</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="F6" s="0" t="s">
         <x:v>36</x:v>
       </x:c>
       <x:c r="G6" s="0" t="s">
-        <x:v>34</x:v>
+        <x:v>37</x:v>
       </x:c>
       <x:c r="H6" s="0" t="s">
-        <x:v>13</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="I6" s="0" t="s">
         <x:v>35</x:v>
@@ -1142,28 +1102,28 @@
     </x:row>
     <x:row r="7" spans="1:10">
       <x:c r="A7" s="0" t="s">
-        <x:v>37</x:v>
+        <x:v>38</x:v>
       </x:c>
       <x:c r="B7" s="0" t="s">
+        <x:v>39</x:v>
+      </x:c>
+      <x:c r="C7" s="0" t="s">
         <x:v>40</x:v>
-      </x:c>
-      <x:c r="C7" s="0" t="s">
-        <x:v>38</x:v>
       </x:c>
       <x:c r="D7" s="0" t="s">
         <x:v>41</x:v>
       </x:c>
       <x:c r="E7" s="0" t="s">
-        <x:v>10</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="F7" s="0" t="s">
         <x:v>42</x:v>
       </x:c>
       <x:c r="G7" s="0" t="s">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="H7" s="0" t="s">
         <x:v>39</x:v>
-      </x:c>
-      <x:c r="H7" s="0" t="s">
-        <x:v>40</x:v>
       </x:c>
       <x:c r="I7" s="0" t="s">
         <x:v>41</x:v>
@@ -1177,383 +1137,383 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="B8" s="0" t="s">
-        <x:v>43</x:v>
+        <x:v>44</x:v>
       </x:c>
       <x:c r="C8" s="0" t="s">
-        <x:v>10</x:v>
+        <x:v>45</x:v>
       </x:c>
       <x:c r="D8" s="0" t="s">
-        <x:v>10</x:v>
+        <x:v>46</x:v>
       </x:c>
       <x:c r="E8" s="0" t="s">
-        <x:v>10</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="F8" s="0" t="s">
-        <x:v>10</x:v>
+        <x:v>47</x:v>
       </x:c>
       <x:c r="G8" s="0" t="s">
-        <x:v>10</x:v>
+        <x:v>48</x:v>
       </x:c>
       <x:c r="H8" s="0" t="s">
-        <x:v>43</x:v>
+        <x:v>44</x:v>
       </x:c>
       <x:c r="I8" s="0" t="s">
-        <x:v>10</x:v>
+        <x:v>46</x:v>
       </x:c>
       <x:c r="J8" s="0" t="s">
-        <x:v>10</x:v>
+        <x:v>47</x:v>
       </x:c>
     </x:row>
     <x:row r="9" spans="1:10">
       <x:c r="A9" s="0" t="s">
-        <x:v>9</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="B9" s="0" t="s">
-        <x:v>46</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="C9" s="0" t="s">
-        <x:v>44</x:v>
+        <x:v>51</x:v>
       </x:c>
       <x:c r="D9" s="0" t="s">
-        <x:v>47</x:v>
+        <x:v>52</x:v>
       </x:c>
       <x:c r="E9" s="0" t="s">
-        <x:v>10</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="F9" s="0" t="s">
-        <x:v>48</x:v>
+        <x:v>53</x:v>
       </x:c>
       <x:c r="G9" s="0" t="s">
-        <x:v>45</x:v>
+        <x:v>54</x:v>
       </x:c>
       <x:c r="H9" s="0" t="s">
-        <x:v>46</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="I9" s="0" t="s">
-        <x:v>47</x:v>
+        <x:v>52</x:v>
       </x:c>
       <x:c r="J9" s="0" t="s">
-        <x:v>48</x:v>
+        <x:v>53</x:v>
       </x:c>
     </x:row>
     <x:row r="10" spans="1:10">
       <x:c r="A10" s="0" t="s">
-        <x:v>49</x:v>
+        <x:v>23</x:v>
       </x:c>
       <x:c r="B10" s="0" t="s">
-        <x:v>52</x:v>
+        <x:v>55</x:v>
       </x:c>
       <x:c r="C10" s="0" t="s">
-        <x:v>50</x:v>
+        <x:v>56</x:v>
       </x:c>
       <x:c r="D10" s="0" t="s">
-        <x:v>53</x:v>
+        <x:v>57</x:v>
       </x:c>
       <x:c r="E10" s="0" t="s">
-        <x:v>10</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="F10" s="0" t="s">
-        <x:v>54</x:v>
+        <x:v>58</x:v>
       </x:c>
       <x:c r="G10" s="0" t="s">
-        <x:v>51</x:v>
+        <x:v>59</x:v>
       </x:c>
       <x:c r="H10" s="0" t="s">
-        <x:v>52</x:v>
+        <x:v>55</x:v>
       </x:c>
       <x:c r="I10" s="0" t="s">
-        <x:v>53</x:v>
+        <x:v>57</x:v>
       </x:c>
       <x:c r="J10" s="0" t="s">
-        <x:v>54</x:v>
+        <x:v>58</x:v>
       </x:c>
     </x:row>
     <x:row r="11" spans="1:10">
       <x:c r="A11" s="0" t="s">
-        <x:v>22</x:v>
+        <x:v>60</x:v>
       </x:c>
       <x:c r="B11" s="0" t="s">
-        <x:v>57</x:v>
+        <x:v>61</x:v>
       </x:c>
       <x:c r="C11" s="0" t="s">
-        <x:v>55</x:v>
+        <x:v>62</x:v>
       </x:c>
       <x:c r="D11" s="0" t="s">
-        <x:v>58</x:v>
+        <x:v>63</x:v>
       </x:c>
       <x:c r="E11" s="0" t="s">
-        <x:v>10</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="F11" s="0" t="s">
-        <x:v>59</x:v>
+        <x:v>64</x:v>
       </x:c>
       <x:c r="G11" s="0" t="s">
-        <x:v>56</x:v>
+        <x:v>65</x:v>
       </x:c>
       <x:c r="H11" s="0" t="s">
-        <x:v>57</x:v>
+        <x:v>61</x:v>
       </x:c>
       <x:c r="I11" s="0" t="s">
-        <x:v>58</x:v>
+        <x:v>63</x:v>
       </x:c>
       <x:c r="J11" s="0" t="s">
-        <x:v>59</x:v>
+        <x:v>64</x:v>
       </x:c>
     </x:row>
     <x:row r="12" spans="1:10">
       <x:c r="A12" s="0" t="s">
-        <x:v>60</x:v>
+        <x:v>66</x:v>
       </x:c>
       <x:c r="B12" s="0" t="s">
-        <x:v>63</x:v>
+        <x:v>67</x:v>
       </x:c>
       <x:c r="C12" s="0" t="s">
-        <x:v>61</x:v>
+        <x:v>68</x:v>
       </x:c>
       <x:c r="D12" s="0" t="s">
-        <x:v>64</x:v>
+        <x:v>69</x:v>
       </x:c>
       <x:c r="E12" s="0" t="s">
-        <x:v>10</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="F12" s="0" t="s">
-        <x:v>65</x:v>
+        <x:v>70</x:v>
       </x:c>
       <x:c r="G12" s="0" t="s">
-        <x:v>62</x:v>
+        <x:v>71</x:v>
       </x:c>
       <x:c r="H12" s="0" t="s">
-        <x:v>63</x:v>
+        <x:v>67</x:v>
       </x:c>
       <x:c r="I12" s="0" t="s">
-        <x:v>64</x:v>
+        <x:v>69</x:v>
       </x:c>
       <x:c r="J12" s="0" t="s">
-        <x:v>65</x:v>
+        <x:v>70</x:v>
       </x:c>
     </x:row>
     <x:row r="13" spans="1:10">
       <x:c r="A13" s="0" t="s">
-        <x:v>66</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="B13" s="0" t="s">
-        <x:v>69</x:v>
+        <x:v>72</x:v>
       </x:c>
       <x:c r="C13" s="0" t="s">
-        <x:v>67</x:v>
+        <x:v>51</x:v>
       </x:c>
       <x:c r="D13" s="0" t="s">
-        <x:v>70</x:v>
+        <x:v>73</x:v>
       </x:c>
       <x:c r="E13" s="0" t="s">
-        <x:v>10</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="F13" s="0" t="s">
-        <x:v>71</x:v>
+        <x:v>74</x:v>
       </x:c>
       <x:c r="G13" s="0" t="s">
-        <x:v>68</x:v>
+        <x:v>75</x:v>
       </x:c>
       <x:c r="H13" s="0" t="s">
-        <x:v>69</x:v>
+        <x:v>72</x:v>
       </x:c>
       <x:c r="I13" s="0" t="s">
-        <x:v>70</x:v>
+        <x:v>73</x:v>
       </x:c>
       <x:c r="J13" s="0" t="s">
-        <x:v>71</x:v>
+        <x:v>74</x:v>
       </x:c>
     </x:row>
     <x:row r="14" spans="1:10">
       <x:c r="A14" s="0" t="s">
-        <x:v>72</x:v>
+        <x:v>60</x:v>
       </x:c>
       <x:c r="B14" s="0" t="s">
-        <x:v>75</x:v>
+        <x:v>76</x:v>
       </x:c>
       <x:c r="C14" s="0" t="s">
-        <x:v>73</x:v>
+        <x:v>77</x:v>
       </x:c>
       <x:c r="D14" s="0" t="s">
+        <x:v>78</x:v>
+      </x:c>
+      <x:c r="E14" s="0" t="s">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="F14" s="0" t="s">
+        <x:v>79</x:v>
+      </x:c>
+      <x:c r="G14" s="0" t="s">
+        <x:v>80</x:v>
+      </x:c>
+      <x:c r="H14" s="0" t="s">
         <x:v>76</x:v>
       </x:c>
-      <x:c r="E14" s="0" t="s">
-        <x:v>10</x:v>
-      </x:c>
-      <x:c r="F14" s="0" t="s">
-        <x:v>77</x:v>
-      </x:c>
-      <x:c r="G14" s="0" t="s">
-        <x:v>74</x:v>
-      </x:c>
-      <x:c r="H14" s="0" t="s">
-        <x:v>75</x:v>
-      </x:c>
       <x:c r="I14" s="0" t="s">
-        <x:v>76</x:v>
+        <x:v>78</x:v>
       </x:c>
       <x:c r="J14" s="0" t="s">
-        <x:v>77</x:v>
+        <x:v>79</x:v>
       </x:c>
     </x:row>
     <x:row r="15" spans="1:10">
       <x:c r="A15" s="0" t="s">
-        <x:v>9</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="B15" s="0" t="s">
-        <x:v>79</x:v>
+        <x:v>81</x:v>
       </x:c>
       <x:c r="C15" s="0" t="s">
-        <x:v>50</x:v>
+        <x:v>82</x:v>
       </x:c>
       <x:c r="D15" s="0" t="s">
-        <x:v>80</x:v>
+        <x:v>83</x:v>
       </x:c>
       <x:c r="E15" s="0" t="s">
-        <x:v>10</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="F15" s="0" t="s">
+        <x:v>84</x:v>
+      </x:c>
+      <x:c r="G15" s="0" t="s">
+        <x:v>85</x:v>
+      </x:c>
+      <x:c r="H15" s="0" t="s">
         <x:v>81</x:v>
       </x:c>
-      <x:c r="G15" s="0" t="s">
-        <x:v>78</x:v>
-      </x:c>
-      <x:c r="H15" s="0" t="s">
-        <x:v>79</x:v>
-      </x:c>
       <x:c r="I15" s="0" t="s">
-        <x:v>80</x:v>
+        <x:v>83</x:v>
       </x:c>
       <x:c r="J15" s="0" t="s">
-        <x:v>81</x:v>
+        <x:v>84</x:v>
       </x:c>
     </x:row>
     <x:row r="16" spans="1:10">
       <x:c r="A16" s="0" t="s">
-        <x:v>66</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="B16" s="0" t="s">
-        <x:v>84</x:v>
+        <x:v>86</x:v>
       </x:c>
       <x:c r="C16" s="0" t="s">
-        <x:v>82</x:v>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="D16" s="0" t="s">
-        <x:v>85</x:v>
+        <x:v>87</x:v>
       </x:c>
       <x:c r="E16" s="0" t="s">
-        <x:v>10</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="F16" s="0" t="s">
+        <x:v>88</x:v>
+      </x:c>
+      <x:c r="G16" s="0" t="s">
+        <x:v>89</x:v>
+      </x:c>
+      <x:c r="H16" s="0" t="s">
         <x:v>86</x:v>
       </x:c>
-      <x:c r="G16" s="0" t="s">
-        <x:v>83</x:v>
-      </x:c>
-      <x:c r="H16" s="0" t="s">
-        <x:v>84</x:v>
-      </x:c>
       <x:c r="I16" s="0" t="s">
-        <x:v>85</x:v>
+        <x:v>87</x:v>
       </x:c>
       <x:c r="J16" s="0" t="s">
-        <x:v>86</x:v>
+        <x:v>88</x:v>
       </x:c>
     </x:row>
     <x:row r="17" spans="1:10">
       <x:c r="A17" s="0" t="s">
-        <x:v>49</x:v>
+        <x:v>90</x:v>
       </x:c>
       <x:c r="B17" s="0" t="s">
-        <x:v>89</x:v>
+        <x:v>91</x:v>
       </x:c>
       <x:c r="C17" s="0" t="s">
-        <x:v>87</x:v>
+        <x:v>92</x:v>
       </x:c>
       <x:c r="D17" s="0" t="s">
-        <x:v>90</x:v>
+        <x:v>93</x:v>
       </x:c>
       <x:c r="E17" s="0" t="s">
-        <x:v>10</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="F17" s="0" t="s">
+        <x:v>94</x:v>
+      </x:c>
+      <x:c r="G17" s="0" t="s">
+        <x:v>95</x:v>
+      </x:c>
+      <x:c r="H17" s="0" t="s">
         <x:v>91</x:v>
       </x:c>
-      <x:c r="G17" s="0" t="s">
-        <x:v>88</x:v>
-      </x:c>
-      <x:c r="H17" s="0" t="s">
-        <x:v>89</x:v>
-      </x:c>
       <x:c r="I17" s="0" t="s">
-        <x:v>90</x:v>
+        <x:v>93</x:v>
       </x:c>
       <x:c r="J17" s="0" t="s">
-        <x:v>91</x:v>
+        <x:v>94</x:v>
       </x:c>
     </x:row>
     <x:row r="18" spans="1:10">
       <x:c r="A18" s="0" t="s">
-        <x:v>9</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="B18" s="0" t="s">
-        <x:v>93</x:v>
+        <x:v>96</x:v>
       </x:c>
       <x:c r="C18" s="0" t="s">
-        <x:v>38</x:v>
+        <x:v>97</x:v>
       </x:c>
       <x:c r="D18" s="0" t="s">
-        <x:v>94</x:v>
+        <x:v>98</x:v>
       </x:c>
       <x:c r="E18" s="0" t="s">
-        <x:v>10</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="F18" s="0" t="s">
-        <x:v>95</x:v>
+        <x:v>99</x:v>
       </x:c>
       <x:c r="G18" s="0" t="s">
-        <x:v>92</x:v>
+        <x:v>100</x:v>
       </x:c>
       <x:c r="H18" s="0" t="s">
-        <x:v>93</x:v>
+        <x:v>96</x:v>
       </x:c>
       <x:c r="I18" s="0" t="s">
-        <x:v>94</x:v>
+        <x:v>98</x:v>
       </x:c>
       <x:c r="J18" s="0" t="s">
-        <x:v>95</x:v>
+        <x:v>99</x:v>
       </x:c>
     </x:row>
     <x:row r="19" spans="1:10">
       <x:c r="A19" s="0" t="s">
-        <x:v>96</x:v>
+        <x:v>90</x:v>
       </x:c>
       <x:c r="B19" s="0" t="s">
-        <x:v>99</x:v>
+        <x:v>91</x:v>
       </x:c>
       <x:c r="C19" s="0" t="s">
-        <x:v>97</x:v>
+        <x:v>92</x:v>
       </x:c>
       <x:c r="D19" s="0" t="s">
-        <x:v>100</x:v>
+        <x:v>93</x:v>
       </x:c>
       <x:c r="E19" s="0" t="s">
-        <x:v>10</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="F19" s="0" t="s">
-        <x:v>101</x:v>
+        <x:v>94</x:v>
       </x:c>
       <x:c r="G19" s="0" t="s">
-        <x:v>98</x:v>
+        <x:v>95</x:v>
       </x:c>
       <x:c r="H19" s="0" t="s">
-        <x:v>99</x:v>
+        <x:v>91</x:v>
       </x:c>
       <x:c r="I19" s="0" t="s">
-        <x:v>100</x:v>
+        <x:v>93</x:v>
       </x:c>
       <x:c r="J19" s="0" t="s">
-        <x:v>101</x:v>
+        <x:v>94</x:v>
       </x:c>
     </x:row>
     <x:row r="20" spans="1:10">
@@ -1561,31 +1521,31 @@
         <x:v>49</x:v>
       </x:c>
       <x:c r="B20" s="0" t="s">
-        <x:v>104</x:v>
+        <x:v>96</x:v>
       </x:c>
       <x:c r="C20" s="0" t="s">
-        <x:v>102</x:v>
+        <x:v>97</x:v>
       </x:c>
       <x:c r="D20" s="0" t="s">
-        <x:v>105</x:v>
+        <x:v>98</x:v>
       </x:c>
       <x:c r="E20" s="0" t="s">
-        <x:v>10</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="F20" s="0" t="s">
-        <x:v>106</x:v>
+        <x:v>99</x:v>
       </x:c>
       <x:c r="G20" s="0" t="s">
-        <x:v>103</x:v>
+        <x:v>100</x:v>
       </x:c>
       <x:c r="H20" s="0" t="s">
-        <x:v>104</x:v>
+        <x:v>96</x:v>
       </x:c>
       <x:c r="I20" s="0" t="s">
-        <x:v>105</x:v>
+        <x:v>98</x:v>
       </x:c>
       <x:c r="J20" s="0" t="s">
-        <x:v>106</x:v>
+        <x:v>99</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>